<commit_message>
Every SKU with no RRP is named before the slow part, not after it
</commit_message>
<xml_diff>
--- a/Claude outputs/Brook St Quarantine Master File 14.09.26.xlsx
+++ b/Claude outputs/Brook St Quarantine Master File 14.09.26.xlsx
@@ -2450,7 +2450,11 @@
           <t>Pink</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
           <t>ZIM CRUSH FLOWER LS RUFFLE HEM PRINT MINI DRESS PINK</t>
@@ -2713,6 +2717,9 @@
         <is>
           <t>MAGDA B RE26 T SHIRT 01 PINK</t>
         </is>
+      </c>
+      <c r="K27" t="n">
+        <v>500</v>
       </c>
       <c r="L27" t="n">
         <v>1</v>

</xml_diff>